<commit_message>
feat(ui+presentation): prominent 3-phase frontend navigation and comprehensive presentation suite update
- Equal 3-column prominent display for all 3 phases in frontend UI (no side scrolling or hidden tabs)
- Interactive 3-phase top navigation strip and clickable hero cards with instant tab switching
- Shortened clean tab labels: Phase 1 Deep Extractor, Phase 2 Meta-Analysis & Synthesis, Phase 3 Research Gap & Thesis Navigator
- Updated PPTX and HTML academic presentations with Slides 13-16 covering Governance, TrialMind/RCTMethodologyIE, Phase 3 5-Pillar Architecture, and Phase 2 20 Supreme Rules
- All 90 tests passing green
</commit_message>
<xml_diff>
--- a/outputs/analysis/Mixed_Metabolic_Cohort/Mixed_Metabolic_Cohort_MANDOROS_Master_Report.xlsx
+++ b/outputs/analysis/Mixed_Metabolic_Cohort/Mixed_Metabolic_Cohort_MANDOROS_Master_Report.xlsx
@@ -13689,7 +13689,7 @@
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
         <is>
-          <t>Adaptation Strategy: Trials evaluate 2 distinct active ingredients (Metformin, Orlistat) with differing measurement endpoints and follow-up horizons. MANDOROS automatically adapted by: (1) Running direct pooling on exact parameter matches where available; (2) Constructing Clinical Outcome Domains and applying scale-free Standardized Mean Differences (Hedges' g) to bridge differing metrics (e.g. BMI vs. Body Weight vs. Waist Circumference); (3) Performing Bucher anchored indirect comparisons against common control arms with SUCRA ranking; and (4) Normalizing durations into monthly rate-of-change trajectories in predictive meta-regression. Specifically, because DPP_Extended_Cohort measured 'primary outcome' over nan nan (Reported in protocol) and DPP_Metformin_2012 measured 'high adherence' over 2.0 years (Metformin 850mg (850.0 mg - experimental); Placebo (nan nan - placebo)), MANDOROS automatically applied Tier 2 Scale-Free Standardized Mean Difference (Hedges' g SMD) and clinical domain bridging (Other Clinical &amp; Laboratory Endpoints) to synthesize their therapeutic impact on a unified, dimensionless scale while computing monthly rate-of-change trajectories to reconcile differing follow-up horizons.</t>
+          <t>Adaptation Strategy: Trials evaluate 2 distinct active ingredients (Metformin, Orlistat) with differing measurement endpoints and follow-up horizons. MANDOROS automatically adapted by: (1) Running direct pooling on exact parameter matches where available; (2) Constructing Clinical Outcome Domains and applying scale-free Standardized Mean Differences (Hedges' g) to bridge differing metrics (e.g. BMI vs. Body Weight vs. Waist Circumference); (3) Performing Bucher anchored indirect comparisons against common control arms with SUCRA ranking; and (4) Normalizing durations into monthly rate-of-change trajectories in predictive meta-regression. Specifically, because DPP_Extended_Cohort measured 'primary outcome' over nan nan (Reported in protocol) and DPP_Metformin_2012 measured 'weight loss &gt;= 5%' over 2.0 years (Metformin 850mg (850.0 mg - experimental); Placebo (nan nan - placebo)), MANDOROS automatically applied Tier 2 Scale-Free Standardized Mean Difference (Hedges' g SMD) and clinical domain bridging (Other Clinical &amp; Laboratory Endpoints) to synthesize their therapeutic impact on a unified, dimensionless scale while computing monthly rate-of-change trajectories to reconcile differing follow-up horizons.</t>
         </is>
       </c>
     </row>
@@ -14235,7 +14235,7 @@
       </c>
       <c r="M6" s="18" t="inlineStr">
         <is>
-          <t>NOT_ESTIMABLE: Domain 'Anthropometric &amp; Weight Management' contains 3 distinct clinical constructs (weight_loss, waist_circumference, bmi). Omnibus pooling of clinically unrelated endpoints into a single SMD is methodologically invalid.</t>
+          <t>NOT_ESTIMABLE: Domain 'Anthropometric &amp; Weight Management' contains 3 distinct clinical constructs (waist_circumference, bmi, weight_loss). Omnibus pooling of clinically unrelated endpoints into a single SMD is methodologically invalid.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(gsap-ui): eliminate tab disfiguring lines, fix wrapping/overlap collision, streamline NCPI banner, and activate GSAP motion architecture
</commit_message>
<xml_diff>
--- a/outputs/analysis/Mixed_Metabolic_Cohort/Mixed_Metabolic_Cohort_MANDOROS_Master_Report.xlsx
+++ b/outputs/analysis/Mixed_Metabolic_Cohort/Mixed_Metabolic_Cohort_MANDOROS_Master_Report.xlsx
@@ -13689,7 +13689,7 @@
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
         <is>
-          <t>Adaptation Strategy: Trials evaluate 2 distinct active ingredients (Metformin, Orlistat) with differing measurement endpoints and follow-up horizons. MANDOROS automatically adapted by: (1) Running direct pooling on exact parameter matches where available; (2) Constructing Clinical Outcome Domains and applying scale-free Standardized Mean Differences (Hedges' g) to bridge differing metrics (e.g. BMI vs. Body Weight vs. Waist Circumference); (3) Performing Bucher anchored indirect comparisons against common control arms with SUCRA ranking; and (4) Normalizing durations into monthly rate-of-change trajectories in predictive meta-regression. Specifically, because DPP_Extended_Cohort measured 'primary outcome' over nan nan (Reported in protocol) and DPP_Metformin_2012 measured 'weight loss &gt;= 5%' over 2.0 years (Metformin 850mg (850.0 mg - experimental); Placebo (nan nan - placebo)), MANDOROS automatically applied Tier 2 Scale-Free Standardized Mean Difference (Hedges' g SMD) and clinical domain bridging (Other Clinical &amp; Laboratory Endpoints) to synthesize their therapeutic impact on a unified, dimensionless scale while computing monthly rate-of-change trajectories to reconcile differing follow-up horizons.</t>
+          <t>Adaptation Strategy: Trials evaluate 2 distinct active ingredients (Metformin, Orlistat) with differing measurement endpoints and follow-up horizons. MANDOROS automatically adapted by: (1) Running direct pooling on exact parameter matches where available; (2) Constructing Clinical Outcome Domains and applying scale-free Standardized Mean Differences (Hedges' g) to bridge differing metrics (e.g. BMI vs. Body Weight vs. Waist Circumference); (3) Performing Bucher anchored indirect comparisons against common control arms with SUCRA ranking; and (4) Normalizing durations into monthly rate-of-change trajectories in predictive meta-regression. Specifically, because DPP_Extended_Cohort measured 'primary outcome' over nan nan (Reported in protocol) and DPP_Metformin_2012 measured 'weight_loss' over 2.0 years (Metformin 850mg (850.0 mg - experimental); Placebo (nan nan - placebo)), MANDOROS automatically applied Tier 2 Scale-Free Standardized Mean Difference (Hedges' g SMD) and clinical domain bridging (Other Clinical &amp; Laboratory Endpoints) to synthesize their therapeutic impact on a unified, dimensionless scale while computing monthly rate-of-change trajectories to reconcile differing follow-up horizons.</t>
         </is>
       </c>
     </row>
@@ -14235,7 +14235,7 @@
       </c>
       <c r="M6" s="18" t="inlineStr">
         <is>
-          <t>NOT_ESTIMABLE: Domain 'Anthropometric &amp; Weight Management' contains 3 distinct clinical constructs (waist_circumference, bmi, weight_loss). Omnibus pooling of clinically unrelated endpoints into a single SMD is methodologically invalid.</t>
+          <t>NOT_ESTIMABLE: Domain 'Anthropometric &amp; Weight Management' contains 3 distinct clinical constructs (waist_circumference, weight_loss, bmi). Omnibus pooling of clinically unrelated endpoints into a single SMD is methodologically invalid.</t>
         </is>
       </c>
     </row>

</xml_diff>